<commit_message>
Edit and delete payments with a change history (version 1.2.1)
Client request: the admin can correct a payment entered wrongly (date,
amount, method, reference, remarks) or delete it, with a reason. The receipt
number stays the same, the amount can never exceed the fee less the other
payments, and every edit and deletion is kept in the new PaymentChange table,
shown with Change History on the Payments screen.

Schema 14 adds the PaymentChange table. From version 1.2 (schema 13) on, an
older database is upgraded in place at start and keeps its data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YAxGRtyyDx6XhwjMNzt5x2
</commit_message>
<xml_diff>
--- a/docs/TestCases.xlsx
+++ b/docs/TestCases.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$J$153</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$J$158</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -673,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J153"/>
+  <dimension ref="A1:J158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1028,27 +1028,27 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Sign in</t>
+          <t>Installation</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Default user name filled in</t>
+          <t>Update from version 1.2 keeps data</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Start the program</t>
+          <t>Install 1.2.1 over 1.2 with students and payments</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>User name shows admin; cursor is in the password box</t>
+          <t>Database upgraded in place; all data kept</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -1073,22 +1073,22 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Correct login</t>
+          <t>Default user name filled in</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Password admin &gt; Sign in</t>
+          <t>Start the program</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Main window opens on the Dashboard</t>
+          <t>User name shows admin; cursor is in the password box</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -1113,17 +1113,17 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Wrong password</t>
+          <t>Correct login</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Enter a wrong password &gt; Sign in</t>
+          <t>Password admin &gt; Sign in</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Message 'Incorrect user name or password'; password box cleared</t>
+          <t>Main window opens on the Dashboard</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
@@ -1153,22 +1153,22 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>User name not case sensitive</t>
+          <t>Wrong password</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>User name ADMIN, correct password</t>
+          <t>Enter a wrong password &gt; Sign in</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Sign in succeeds</t>
+          <t>Message 'Incorrect user name or password'; password box cleared</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -1193,22 +1193,22 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Password is case sensitive</t>
+          <t>User name not case sensitive</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Password ADMIN</t>
+          <t>User name ADMIN, correct password</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>Sign in refused</t>
+          <t>Sign in succeeds</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -1233,17 +1233,17 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Hostel chosen at sign in</t>
+          <t>Password is case sensitive</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>With two hostels, choose the second at sign in</t>
+          <t>Password ADMIN</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>Main window shows the second hostel at the top right</t>
+          <t>Sign in refused</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -1268,27 +1268,27 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Admin Account</t>
+          <t>Sign in</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Save admin email and phone</t>
+          <t>Hostel chosen at sign in</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Settings &gt; Admin Account &gt; enter email and phone &gt; Save</t>
+          <t>With two hostels, choose the second at sign in</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>'Saved.' shown; values kept after restarting</t>
+          <t>Main window shows the second hostel at the top right</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
@@ -1313,22 +1313,22 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Invalid email</t>
+          <t>Save admin email and phone</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Enter 'owner' as email &gt; Save</t>
+          <t>Settings &gt; Admin Account &gt; enter email and phone &gt; Save</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Error 'Please enter a valid email address'</t>
+          <t>'Saved.' shown; values kept after restarting</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -1353,22 +1353,22 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Change password</t>
+          <t>Invalid email</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Current admin, new Balaji@2026 twice &gt; Change Password</t>
+          <t>Enter 'owner' as email &gt; Save</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Success message; next sign in works only with the new password</t>
+          <t>Error 'Please enter a valid email address'</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -1393,17 +1393,17 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Wrong current password</t>
+          <t>Change password</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Wrong current password &gt; Change Password</t>
+          <t>Current admin, new Balaji@2026 twice &gt; Change Password</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Error 'The current password is not correct'</t>
+          <t>Success message; next sign in works only with the new password</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
@@ -1433,22 +1433,22 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Password too short</t>
+          <t>Wrong current password</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>New password abc</t>
+          <t>Wrong current password &gt; Change Password</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>Error 'at least 6 characters'</t>
+          <t>Error 'The current password is not correct'</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -1473,17 +1473,17 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Confirmation differs</t>
+          <t>Password too short</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>New and confirm different</t>
+          <t>New password abc</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Error 'not the same'</t>
+          <t>Error 'at least 6 characters'</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
@@ -1508,27 +1508,27 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Hostels</t>
+          <t>Admin Account</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Add hostel</t>
+          <t>Confirmation differs</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Hostels &gt; Add &gt; name, address, phone &gt; Save</t>
+          <t>New and confirm different</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Hostel listed; appears in the hostel selector</t>
+          <t>Error 'not the same'</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -1553,22 +1553,22 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Name required</t>
+          <t>Add hostel</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Add without a name</t>
+          <t>Hostels &gt; Add &gt; name, address, phone &gt; Save</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Error, nothing saved</t>
+          <t>Hostel listed; appears in the hostel selector</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -1593,17 +1593,17 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Duplicate hostel name</t>
+          <t>Name required</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Add a hostel with an existing name</t>
+          <t>Add without a name</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Error about the duplicate name</t>
+          <t>Error, nothing saved</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
@@ -1633,17 +1633,17 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Default sharing types</t>
+          <t>Duplicate hostel name</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Open Rooms &gt; Add for the new hostel</t>
+          <t>Add a hostel with an existing name</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Single (1 bed), Double (2 beds), Triple (3 beds) offered; no rent asked</t>
+          <t>Error about the duplicate name</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
@@ -1673,22 +1673,22 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Switch hostel</t>
+          <t>Default sharing types</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Choose another hostel at the top right</t>
+          <t>Open Rooms &gt; Add for the new hostel</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Every screen shows only that hostel's data</t>
+          <t>Single (1 bed), Double (2 beds), Triple (3 beds) offered; no rent asked</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -1708,22 +1708,22 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Colleges</t>
+          <t>Hostels</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Add college</t>
+          <t>Switch hostel</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Colleges &gt; Add &gt; name &gt; Save</t>
+          <t>Choose another hostel at the top right</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>College listed for the selected hostel only</t>
+          <t>Every screen shows only that hostel's data</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
@@ -1753,22 +1753,22 @@
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Duplicate college in same hostel</t>
+          <t>Add college</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Add the same college name again</t>
+          <t>Colleges &gt; Add &gt; name &gt; Save</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Error about the duplicate</t>
+          <t>College listed for the selected hostel only</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
@@ -1793,22 +1793,22 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Delete college in use</t>
+          <t>Duplicate college in same hostel</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Delete a college that has students</t>
+          <t>Add the same college name again</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Refused with a clear message</t>
+          <t>Error about the duplicate</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
@@ -1828,27 +1828,27 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Rooms</t>
+          <t>Colleges</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>No rent on rooms</t>
+          <t>Delete college in use</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Open Rooms</t>
+          <t>Delete a college that has students</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>No rent panel or rent column; sharing type only sets the number of beds</t>
+          <t>Refused with a clear message</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
@@ -1873,17 +1873,17 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Add room</t>
+          <t>No rent on rooms</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Add room 101, Double, Boys</t>
+          <t>Open Rooms</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Room listed with 2 beds, 0 occupied, 2 free</t>
+          <t>No rent panel or rent column; sharing type only sets the number of beds</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
@@ -1913,22 +1913,22 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Duplicate room number</t>
+          <t>Add room</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Add room 101 again (any case)</t>
+          <t>Add room 101, Double, Boys</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Error about the duplicate</t>
+          <t>Room listed with 2 beds, 0 occupied, 2 free</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G31" s="10" t="inlineStr">
@@ -1953,22 +1953,22 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Room for boys or girls required</t>
+          <t>Duplicate room number</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Add a room without choosing Boys/Girls</t>
+          <t>Add room 101 again (any case)</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Error about the duplicate</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G32" s="10" t="inlineStr">
@@ -1993,22 +1993,22 @@
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Reduce sharing below occupancy</t>
+          <t>Room for boys or girls required</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Room with 2 students &gt; change to Single</t>
+          <t>Add a room without choosing Boys/Girls</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Refused</t>
+          <t>Error</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G33" s="10" t="inlineStr">
@@ -2033,12 +2033,12 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Change gender of occupied room</t>
+          <t>Reduce sharing below occupancy</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Occupied boys room &gt; change to Girls</t>
+          <t>Room with 2 students &gt; change to Single</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
@@ -2073,12 +2073,12 @@
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Deactivate occupied room</t>
+          <t>Change gender of occupied room</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Occupied room &gt; untick Active</t>
+          <t>Occupied boys room &gt; change to Girls</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G35" s="10" t="inlineStr">
@@ -2113,17 +2113,17 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Delete room</t>
+          <t>Deactivate occupied room</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Delete a room never used / a room with past students</t>
+          <t>Occupied room &gt; untick Active</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Unused room deleted; used room refused</t>
+          <t>Refused</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
@@ -2148,27 +2148,27 @@
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>Students</t>
+          <t>Rooms</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Add student with required fields</t>
+          <t>Delete room</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Students &gt; Add &gt; name, gender, mobile, college, admission date, father's name and mobile &gt; Save</t>
+          <t>Delete a room never used / a room with past students</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Student listed as Active</t>
+          <t>Unused room deleted; used room refused</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G37" s="10" t="inlineStr">
@@ -2193,17 +2193,17 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Required fields</t>
+          <t>Add student with required fields</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Save without name / mobile / admission date / father's name / father's mobile</t>
+          <t>Students &gt; Add &gt; name, gender, mobile, college, admission date, father's name and mobile &gt; Save</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Clear error for each missing field; nothing saved</t>
+          <t>Student listed as Active</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
@@ -2233,22 +2233,22 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Invalid mobile or email</t>
+          <t>Required fields</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Mobile 12ab, father's email 'abc', mother's mobile 12ab</t>
+          <t>Save without name / mobile / admission date / father's name / father's mobile</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Errors shown</t>
+          <t>Clear error for each missing field; nothing saved</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G39" s="10" t="inlineStr">
@@ -2273,17 +2273,17 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Aadhaar check</t>
+          <t>Invalid mobile or email</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Enter 2345 6789 0124 (valid) and 2345 6789 0123 (invalid)</t>
+          <t>Mobile 12ab, father's email 'abc', mother's mobile 12ab</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Valid one saved; invalid one refused</t>
+          <t>Errors shown</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
@@ -2313,22 +2313,22 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Aadhaar masked</t>
+          <t>Aadhaar check</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>View student list and reports</t>
+          <t>Enter 2345 6789 0124 (valid) and 2345 6789 0123 (invalid)</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Aadhaar shown as XXXX XXXX 0124 only</t>
+          <t>Valid one saved; invalid one refused</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G41" s="10" t="inlineStr">
@@ -2353,22 +2353,22 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Photo and Aadhaar card</t>
+          <t>Aadhaar masked</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Add a JPG photo and a PDF Aadhaar card</t>
+          <t>View student list and reports</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Photo shown; files saved in Photos/Documents</t>
+          <t>Aadhaar shown as XXXX XXXX 0124 only</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G42" s="10" t="inlineStr">
@@ -2393,22 +2393,22 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>File too large or wrong type</t>
+          <t>Photo and Aadhaar card</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Add a 6 MB photo or a .txt file</t>
+          <t>Add a JPG photo and a PDF Aadhaar card</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Refused before saving</t>
+          <t>Photo shown; files saved in Photos/Documents</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G43" s="10" t="inlineStr">
@@ -2433,22 +2433,22 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Search and filters</t>
+          <t>File too large or wrong type</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Type part of a student, father or mother name or mobile; filter by college, course, class, status</t>
+          <t>Add a 6 MB photo or a .txt file</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>List narrows correctly</t>
+          <t>Refused before saving</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G44" s="10" t="inlineStr">
@@ -2473,17 +2473,17 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Edit student</t>
+          <t>Search and filters</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>View / Edit &gt; change mobile &gt; Save</t>
+          <t>Type part of a student, father or mother name or mobile; filter by college, course, class, status</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Change saved</t>
+          <t>List narrows correctly</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
@@ -2513,17 +2513,17 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Delete student with history</t>
+          <t>Edit student</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Delete a student who had a room or invoice</t>
+          <t>View / Edit &gt; change mobile &gt; Save</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Refused</t>
+          <t>Change saved</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
@@ -2553,22 +2553,22 @@
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Father and mother details</t>
+          <t>Delete student with history</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Father &amp; Mother tab: father name, mobile, email; mother name, mobile, email &gt; Save</t>
+          <t>Delete a student who had a room or invoice</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>All six values kept; Father and Father mobile shown in the list</t>
+          <t>Refused</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G47" s="10" t="inlineStr">
@@ -2593,22 +2593,22 @@
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Only father details</t>
+          <t>Father and mother details</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Leave father email and all mother fields empty &gt; Save</t>
+          <t>Father &amp; Mother tab: father name, mobile, email; mother name, mobile, email &gt; Save</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Saved (only father name and mobile are required)</t>
+          <t>All six values kept; Father and Father mobile shown in the list</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G48" s="10" t="inlineStr">
@@ -2633,22 +2633,22 @@
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Take photo with webcam</t>
+          <t>Only father details</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Photo &amp; Aadhaar &gt; Take Photo &gt; Capture &gt; Use Photo &gt; Save</t>
+          <t>Leave father email and all mother fields empty &gt; Save</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Live picture shown; captured photo saved with the student</t>
+          <t>Saved (only father name and mobile are required)</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G49" s="10" t="inlineStr">
@@ -2673,22 +2673,22 @@
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Retake photo</t>
+          <t>Take photo with webcam</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Take Photo &gt; Capture &gt; Retake &gt; Capture &gt; Use Photo</t>
+          <t>Photo &amp; Aadhaar &gt; Take Photo &gt; Capture &gt; Use Photo &gt; Save</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>The second picture is used</t>
+          <t>Live picture shown; captured photo saved with the student</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G50" s="10" t="inlineStr">
@@ -2713,22 +2713,22 @@
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>No camera / camera blocked</t>
+          <t>Retake photo</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Take Photo on a PC without camera, or with camera access off in Windows</t>
+          <t>Take Photo &gt; Capture &gt; Retake &gt; Capture &gt; Use Photo</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Clear message (connect a camera / switch on camera access); Choose Photo still works</t>
+          <t>The second picture is used</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G51" s="10" t="inlineStr">
@@ -2753,22 +2753,22 @@
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>Student I-card</t>
+          <t>No camera / camera blocked</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Select a student &gt; I-Card &gt; Save</t>
+          <t>Take Photo on a PC without camera, or with camera access off in Windows</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>PDF opens: card with photo, name, father, college, room and bed, mobiles, valid till 30 Jun</t>
+          <t>Clear message (connect a camera / switch on camera access); Choose Photo still works</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G52" s="10" t="inlineStr">
@@ -2793,22 +2793,22 @@
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>I-cards for several students</t>
+          <t>Student I-card</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Select 9 students (Ctrl/Shift) &gt; I-Card</t>
+          <t>Select a student &gt; I-Card &gt; Save</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>8 cards on page 1, 1 on page 2</t>
+          <t>PDF opens: card with photo, name, father, college, room and bed, mobiles, valid till 30 Jun</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G53" s="10" t="inlineStr">
@@ -2833,22 +2833,22 @@
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Transport I-card</t>
+          <t>I-cards for several students</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Select a student with transport and one without &gt; Transport I-Card</t>
+          <t>Select 9 students (Ctrl/Shift) &gt; I-Card</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Transport pass only for the student with transport; message names the other</t>
+          <t>8 cards on page 1, 1 on page 2</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G54" s="10" t="inlineStr">
@@ -2873,22 +2873,22 @@
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>I-card without photo</t>
+          <t>Transport I-card</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>I-Card for a student without photo</t>
+          <t>Select a student with transport and one without &gt; Transport I-Card</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Card with empty photo box; message names the student</t>
+          <t>Transport pass only for the student with transport; message names the other</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G55" s="10" t="inlineStr">
@@ -2913,17 +2913,17 @@
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>I-card for student who left</t>
+          <t>I-card without photo</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>I-Card for a student with status Left</t>
+          <t>I-Card for a student without photo</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>No card; message 'has left the hostel'</t>
+          <t>Card with empty photo box; message names the student</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
@@ -2948,27 +2948,27 @@
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>Room Allocation</t>
+          <t>Students</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Check-in with yearly fee</t>
+          <t>I-card for student who left</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Room Allocation &gt; Check-in &gt; student, room 101 &gt; rent 50000, transport 12000 &gt; Check-in</t>
+          <t>I-Card for a student with status Left</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Bed 1 suggested; student in room 101 bed 1; total 62000 shown; invoice for this academic year created</t>
+          <t>No card; message 'has left the hostel'</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G57" s="10" t="inlineStr">
@@ -2993,22 +2993,22 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Choose another bed</t>
+          <t>Check-in with yearly fee</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Check-in a second student, choose bed 2</t>
+          <t>Room Allocation &gt; Check-in &gt; student, room 101 &gt; rent 50000, transport 12000 &gt; Check-in</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Saved in bed 2</t>
+          <t>Bed 1 suggested; student in room 101 bed 1; total 62000 shown; invoice for this academic year created</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G58" s="10" t="inlineStr">
@@ -3033,22 +3033,22 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Only matching rooms offered</t>
+          <t>Choose another bed</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Check in a girl student</t>
+          <t>Check-in a second student, choose bed 2</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Only girls' rooms with a free bed listed</t>
+          <t>Saved in bed 2</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G59" s="10" t="inlineStr">
@@ -3073,17 +3073,17 @@
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>Full room</t>
+          <t>Only matching rooms offered</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Try to fill a room beyond its beds</t>
+          <t>Check in a girl student</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Full room not offered / refused</t>
+          <t>Only girls' rooms with a free bed listed</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
@@ -3113,22 +3113,22 @@
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>Check-in before admission date</t>
+          <t>Full room</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Check-in date earlier than admission date</t>
+          <t>Try to fill a room beyond its beds</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Refused</t>
+          <t>Full room not offered / refused</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G61" s="10" t="inlineStr">
@@ -3153,17 +3153,17 @@
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>Future date</t>
+          <t>Check-in before admission date</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Check-in date in the future</t>
+          <t>Check-in date earlier than admission date</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Not possible</t>
+          <t>Refused</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
@@ -3193,22 +3193,22 @@
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>Transfer</t>
+          <t>Future date</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Transfer &gt; new room and bed &gt; confirm</t>
+          <t>Check-in date in the future</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Old stay closed as Transferred, new stay current, same day</t>
+          <t>Not possible</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G63" s="10" t="inlineStr">
@@ -3233,17 +3233,17 @@
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>Check-out</t>
+          <t>Transfer</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Check-out &gt; confirm</t>
+          <t>Transfer &gt; new room and bed &gt; confirm</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Stay closed; student status Left; bed free</t>
+          <t>Old stay closed as Transferred, new stay current, same day</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
@@ -3273,22 +3273,22 @@
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>Agreement offered after check-in</t>
+          <t>Check-out</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Complete a check-in</t>
+          <t>Check-out &gt; confirm</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Program offers to create the agreement PDF</t>
+          <t>Stay closed; student status Left; bed free</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G65" s="10" t="inlineStr">
@@ -3313,22 +3313,22 @@
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>Rent required at check-in</t>
+          <t>Agreement offered after check-in</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Check-in with the rent empty or 0</t>
+          <t>Complete a check-in</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Refused: enter the room rent for the year; nothing saved</t>
+          <t>Program offers to create the agreement PDF</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G66" s="10" t="inlineStr">
@@ -3353,17 +3353,17 @@
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>Different fees in one room</t>
+          <t>Rent required at check-in</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Check in two students to the same Double room with rent 50000 and 45000</t>
+          <t>Check-in with the rent empty or 0</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Each student's invoice has his own amount</t>
+          <t>Refused: enter the room rent for the year; nothing saved</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
@@ -3393,22 +3393,22 @@
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>Student who already has a fee</t>
+          <t>Different fees in one room</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Check in again a student who already has this year's fee</t>
+          <t>Check in two students to the same Double room with rent 50000 and 45000</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Fee boxes locked showing the existing invoice; no second invoice</t>
+          <t>Each student's invoice has his own amount</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G68" s="10" t="inlineStr">
@@ -3433,17 +3433,17 @@
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Transfer and check-out keep the fee</t>
+          <t>Student who already has a fee</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Transfer, then check out a student</t>
+          <t>Check in again a student who already has this year's fee</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Invoice amounts unchanged; pending still due</t>
+          <t>Fee boxes locked showing the existing invoice; no second invoice</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
@@ -3468,27 +3468,27 @@
       </c>
       <c r="B70" s="9" t="inlineStr">
         <is>
-          <t>Agreement</t>
+          <t>Room Allocation</t>
         </is>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>Create agreement PDF</t>
+          <t>Transfer and check-out keep the fee</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Students &gt; select &gt; Agreement PDF &gt; Save</t>
+          <t>Transfer, then check out a student</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>PDF opens: name, S/o or D/o + father, address, Boys/Girls hostel, room, bed, beds in room, check-in date, annual fee in figures and words</t>
+          <t>Invoice amounts unchanged; pending still due</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G70" s="10" t="inlineStr">
@@ -3513,17 +3513,17 @@
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>Annual fee with transport</t>
+          <t>Create agreement PDF</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Student with rent 120000 and transport 18000 at check-in</t>
+          <t>Students &gt; select &gt; Agreement PDF &gt; Save</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Annual fee Rs. 1,38,000/- (Rupees One Lakh Thirty Eight Thousand Only)</t>
+          <t>PDF opens: name, S/o or D/o + father, address, Boys/Girls hostel, room, bed, beds in room, check-in date, annual fee in figures and words</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
@@ -3553,22 +3553,22 @@
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>Girl student</t>
+          <t>Annual fee with transport</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Agreement for a girl</t>
+          <t>Student with rent 120000 and transport 18000 at check-in</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>D/o and 'Girls Hostel'</t>
+          <t>Annual fee Rs. 1,38,000/- (Rupees One Lakh Thirty Eight Thousand Only)</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G72" s="10" t="inlineStr">
@@ -3593,22 +3593,22 @@
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>No address</t>
+          <t>Girl student</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Student without address</t>
+          <t>Agreement for a girl</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Dotted line after R/o</t>
+          <t>D/o and 'Girls Hostel'</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G73" s="10" t="inlineStr">
@@ -3633,22 +3633,22 @@
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>Student not checked in</t>
+          <t>No address</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Agreement PDF for a student without a room</t>
+          <t>Student without address</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Message to check in first</t>
+          <t>Dotted line after R/o</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G74" s="10" t="inlineStr">
@@ -3673,17 +3673,17 @@
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>Edit agreement text</t>
+          <t>Student not checked in</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Students &gt; Agreement Text &gt; change a rule &gt; Save &gt; create PDF</t>
+          <t>Agreement PDF for a student without a room</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>PDF shows the changed text; Restore Default brings back the original</t>
+          <t>Message to check in first</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
@@ -3713,22 +3713,22 @@
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>Unknown field in text</t>
+          <t>Edit agreement text</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Type {BedNo} in the text &gt; Save</t>
+          <t>Students &gt; Agreement Text &gt; change a rule &gt; Save &gt; create PDF</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Error naming the available fields</t>
+          <t>PDF shows the changed text; Restore Default brings back the original</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G76" s="10" t="inlineStr">
@@ -3748,27 +3748,27 @@
       </c>
       <c r="B77" s="9" t="inlineStr">
         <is>
-          <t>Attendance</t>
+          <t>Agreement</t>
         </is>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>Tonight's sheet</t>
+          <t>Unknown field in text</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Students &gt; Attendance</t>
+          <t>Type {BedNo} in the text &gt; Save</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Today's date; all students in a room tonight with room and bed; all Present; 'Not marked yet'</t>
+          <t>Error naming the available fields</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G77" s="10" t="inlineStr">
@@ -3793,17 +3793,17 @@
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>Mark absent and save</t>
+          <t>Tonight's sheet</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Untick Present for 2 students &gt; Save Attendance</t>
+          <t>Students &gt; Attendance</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>'Saved: x present, 2 absent'; both in the Absent students list</t>
+          <t>Today's date; all students in a room tonight with room and bed; all Present; 'Not marked yet'</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
@@ -3833,17 +3833,17 @@
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>Earlier date</t>
+          <t>Mark absent and save</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Choose yesterday</t>
+          <t>Untick Present for 2 students &gt; Save Attendance</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Yesterday's saved attendance (or all present, not marked)</t>
+          <t>'Saved: x present, 2 absent'; both in the Absent students list</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
@@ -3873,22 +3873,22 @@
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>Correct an earlier date</t>
+          <t>Earlier date</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Change yesterday's attendance &gt; Save</t>
+          <t>Choose yesterday</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Correction saved</t>
+          <t>Yesterday's saved attendance (or all present, not marked)</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G80" s="10" t="inlineStr">
@@ -3913,22 +3913,22 @@
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>Future date</t>
+          <t>Correct an earlier date</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Try to choose tomorrow</t>
+          <t>Change yesterday's attendance &gt; Save</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>Not possible</t>
+          <t>Correction saved</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G81" s="10" t="inlineStr">
@@ -3953,22 +3953,22 @@
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>Unsaved changes</t>
+          <t>Future date</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Change ticks, then pick another date</t>
+          <t>Try to choose tomorrow</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>Asks whether to discard the changes</t>
+          <t>Not possible</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G82" s="10" t="inlineStr">
@@ -3993,17 +3993,17 @@
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>Checked out student</t>
+          <t>Unsaved changes</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Check out a student today</t>
+          <t>Change ticks, then pick another date</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>Not on tonight's sheet; still on earlier nights</t>
+          <t>Asks whether to discard the changes</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
@@ -4033,22 +4033,22 @@
       </c>
       <c r="C84" s="9" t="inlineStr">
         <is>
-          <t>Email parents of absent</t>
+          <t>Checked out student</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Email Parents &gt; confirm</t>
+          <t>Check out a student today</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>Email goes to the mother (father when no mother email); 'Emailed' shown; copy to admin; in Email history</t>
+          <t>Not on tonight's sheet; still on earlier nights</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G84" s="10" t="inlineStr">
@@ -4073,22 +4073,22 @@
       </c>
       <c r="C85" s="9" t="inlineStr">
         <is>
-          <t>Email again</t>
+          <t>Email parents of absent</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Click Email Parents again for the same date</t>
+          <t>Email Parents &gt; confirm</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>Asks before emailing the same parents again</t>
+          <t>Email goes to the mother (father when no mother email); 'Emailed' shown; copy to admin; in Email history</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G85" s="10" t="inlineStr">
@@ -4113,22 +4113,22 @@
       </c>
       <c r="C86" s="9" t="inlineStr">
         <is>
-          <t>No parent email</t>
+          <t>Email again</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Absent student without father or mother email &gt; Email Parents</t>
+          <t>Click Email Parents again for the same date</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>Listed as a problem; others are emailed</t>
+          <t>Asks before emailing the same parents again</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G86" s="10" t="inlineStr">
@@ -4148,27 +4148,27 @@
       </c>
       <c r="B87" s="9" t="inlineStr">
         <is>
-          <t>Invoices</t>
+          <t>Attendance</t>
         </is>
       </c>
       <c r="C87" s="9" t="inlineStr">
         <is>
-          <t>Invoice from check-in</t>
+          <t>No parent email</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>Invoices after a check-in with rent 50000 + transport 12000</t>
+          <t>Absent student without father or mother email &gt; Email Parents</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>Invoice SBH/2026-27/0001, year 2026-27, rent 50000, transport 12000, total 62000, Unpaid</t>
+          <t>Listed as a problem; others are emailed</t>
         </is>
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G87" s="10" t="inlineStr">
@@ -4193,22 +4193,22 @@
       </c>
       <c r="C88" s="9" t="inlineStr">
         <is>
-          <t>Joining mid-year</t>
+          <t>Invoice from check-in</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Check in a student in January</t>
+          <t>Invoices after a check-in with rent 50000 + transport 12000</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>Full yearly fee charged</t>
+          <t>Invoice SBH/2026-27/0001, year 2026-27, rent 50000, transport 12000, total 62000, Unpaid</t>
         </is>
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G88" s="10" t="inlineStr">
@@ -4233,22 +4233,22 @@
       </c>
       <c r="C89" s="9" t="inlineStr">
         <is>
-          <t>Edit fee</t>
+          <t>Joining mid-year</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Select invoice &gt; Edit Fee &gt; transport 0 &gt; Save</t>
+          <t>Check in a student in January</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>Total and pending updated</t>
+          <t>Full yearly fee charged</t>
         </is>
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G89" s="10" t="inlineStr">
@@ -4273,17 +4273,17 @@
       </c>
       <c r="C90" s="9" t="inlineStr">
         <is>
-          <t>Edit fee below paid</t>
+          <t>Edit fee</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Paid 15000 &gt; Edit Fee total 10000</t>
+          <t>Select invoice &gt; Edit Fee &gt; transport 0 &gt; Save</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>Refused: cannot be less than paid</t>
+          <t>Total and pending updated</t>
         </is>
       </c>
       <c r="F90" s="9" t="inlineStr">
@@ -4313,17 +4313,17 @@
       </c>
       <c r="C91" s="9" t="inlineStr">
         <is>
-          <t>New Year Fees</t>
+          <t>Edit fee below paid</t>
         </is>
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>New Year Fees &gt; next year &gt; rent and transport for 2 students &gt; Create Fees</t>
+          <t>Paid 15000 &gt; Edit Fee total 10000</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>2 invoices SBH/next-year/0001, 0002; last year's amounts shown for reference</t>
+          <t>Refused: cannot be less than paid</t>
         </is>
       </c>
       <c r="F91" s="9" t="inlineStr">
@@ -4353,22 +4353,22 @@
       </c>
       <c r="C92" s="9" t="inlineStr">
         <is>
-          <t>New Year Fees skips empty rows</t>
+          <t>New Year Fees</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Leave a student's row empty &gt; Create Fees</t>
+          <t>New Year Fees &gt; next year &gt; rent and transport for 2 students &gt; Create Fees</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>That student gets no fee; others created</t>
+          <t>2 invoices SBH/next-year/0001, 0002; last year's amounts shown for reference</t>
         </is>
       </c>
       <c r="F92" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G92" s="10" t="inlineStr">
@@ -4393,17 +4393,17 @@
       </c>
       <c r="C93" s="9" t="inlineStr">
         <is>
-          <t>New Year Fees wrong amount</t>
+          <t>New Year Fees skips empty rows</t>
         </is>
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>Rent 0 or letters for one student</t>
+          <t>Leave a student's row empty &gt; Create Fees</t>
         </is>
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>Error naming the student; nothing created</t>
+          <t>That student gets no fee; others created</t>
         </is>
       </c>
       <c r="F93" s="9" t="inlineStr">
@@ -4433,17 +4433,17 @@
       </c>
       <c r="C94" s="9" t="inlineStr">
         <is>
-          <t>Numbering</t>
+          <t>New Year Fees wrong amount</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>Create three fees</t>
+          <t>Rent 0 or letters for one student</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>0001, 0002, 0003 in the academic year</t>
+          <t>Error naming the student; nothing created</t>
         </is>
       </c>
       <c r="F94" s="9" t="inlineStr">
@@ -4473,22 +4473,22 @@
       </c>
       <c r="C95" s="9" t="inlineStr">
         <is>
-          <t>View / Print with payments</t>
+          <t>Numbering</t>
         </is>
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>Invoice with two payments &gt; View / Print</t>
+          <t>Create three fees</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr">
         <is>
-          <t>PDF: room rent, transport, total, both payments (date, receipt, method), total paid, pending</t>
+          <t>0001, 0002, 0003 in the academic year</t>
         </is>
       </c>
       <c r="F95" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G95" s="10" t="inlineStr">
@@ -4513,22 +4513,22 @@
       </c>
       <c r="C96" s="9" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>View / Print with payments</t>
         </is>
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>Status Partly paid; Year 2026-27; search a name</t>
+          <t>Invoice with two payments &gt; View / Print</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>List narrows; totals update</t>
+          <t>PDF: room rent, transport, total, both payments (date, receipt, method), total paid, pending</t>
         </is>
       </c>
       <c r="F96" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G96" s="10" t="inlineStr">
@@ -4553,22 +4553,22 @@
       </c>
       <c r="C97" s="9" t="inlineStr">
         <is>
-          <t>Delete invoice</t>
+          <t>Filters</t>
         </is>
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>Delete an invoice without payments / with a payment</t>
+          <t>Status Partly paid; Year 2026-27; search a name</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>Deleted / refused (use Edit Fee)</t>
+          <t>List narrows; totals update</t>
         </is>
       </c>
       <c r="F97" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G97" s="10" t="inlineStr">
@@ -4588,27 +4588,27 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Invoices</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr">
         <is>
-          <t>Part payment</t>
+          <t>Delete invoice</t>
         </is>
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>Fee 62000 &gt; Record Payment 10000 Cash</t>
+          <t>Delete an invoice without payments / with a payment</t>
         </is>
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Receipt SBH/R/2026-27/0001; invoice Partly paid, pending 52000</t>
+          <t>Deleted / refused (use Edit Fee)</t>
         </is>
       </c>
       <c r="F98" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G98" s="10" t="inlineStr">
@@ -4633,17 +4633,17 @@
       </c>
       <c r="C99" s="9" t="inlineStr">
         <is>
-          <t>Further instalments</t>
+          <t>Part payment</t>
         </is>
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>Pay 5000 after 15 days, then the remaining 47000 by UPI</t>
+          <t>Fee 62000 &gt; Record Payment 10000 Cash</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>Pending 47000, then 0; invoice Paid; Record Payment disabled</t>
+          <t>Receipt SBH/R/2026-27/0001; invoice Partly paid, pending 52000</t>
         </is>
       </c>
       <c r="F99" s="9" t="inlineStr">
@@ -4673,17 +4673,17 @@
       </c>
       <c r="C100" s="9" t="inlineStr">
         <is>
-          <t>More than pending</t>
+          <t>Further instalments</t>
         </is>
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>Enter 60000 when 47000 is pending</t>
+          <t>Pay 5000 after 15 days, then the remaining 47000 by UPI</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>Refused (no advance payments)</t>
+          <t>Pending 47000, then 0; invoice Paid; Record Payment disabled</t>
         </is>
       </c>
       <c r="F100" s="9" t="inlineStr">
@@ -4713,17 +4713,17 @@
       </c>
       <c r="C101" s="9" t="inlineStr">
         <is>
-          <t>Reference required</t>
+          <t>More than pending</t>
         </is>
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>Cheque / UPI / Bank transfer without reference</t>
+          <t>Enter 60000 when 47000 is pending</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>Refused</t>
+          <t>Refused (no advance payments)</t>
         </is>
       </c>
       <c r="F101" s="9" t="inlineStr">
@@ -4753,12 +4753,12 @@
       </c>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>Invalid amount</t>
+          <t>Reference required</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>0, negative, 100.555, letters</t>
+          <t>Cheque / UPI / Bank transfer without reference</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="F102" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G102" s="10" t="inlineStr">
@@ -4793,22 +4793,22 @@
       </c>
       <c r="C103" s="9" t="inlineStr">
         <is>
-          <t>Future date</t>
+          <t>Invalid amount</t>
         </is>
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>Payment date tomorrow</t>
+          <t>0, negative, 100.555, letters</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>Not possible</t>
+          <t>Refused</t>
         </is>
       </c>
       <c r="F103" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G103" s="10" t="inlineStr">
@@ -4833,22 +4833,22 @@
       </c>
       <c r="C104" s="9" t="inlineStr">
         <is>
-          <t>Receipt PDF</t>
+          <t>Future date</t>
         </is>
       </c>
       <c r="D104" s="9" t="inlineStr">
         <is>
-          <t>Payments &gt; View / Print</t>
+          <t>Payment date tomorrow</t>
         </is>
       </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>Receipt with amount in words and balance pending</t>
+          <t>Not possible</t>
         </is>
       </c>
       <c r="F104" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G104" s="10" t="inlineStr">
@@ -4873,22 +4873,22 @@
       </c>
       <c r="C105" s="9" t="inlineStr">
         <is>
-          <t>Delete payment</t>
+          <t>Receipt PDF</t>
         </is>
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>Delete a payment &gt; confirm</t>
+          <t>Payments &gt; View / Print</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>Amount pending again on the invoice</t>
+          <t>Receipt with amount in words and balance pending</t>
         </is>
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G105" s="10" t="inlineStr">
@@ -4948,22 +4948,22 @@
       </c>
       <c r="B107" s="9" t="inlineStr">
         <is>
-          <t>Fee Reminders</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="C107" s="9" t="inlineStr">
         <is>
-          <t>List</t>
+          <t>Edit payment</t>
         </is>
       </c>
       <c r="D107" s="9" t="inlineStr">
         <is>
-          <t>Fee Reminders</t>
+          <t>Payments &gt; select &gt; Edit &gt; amount 10000 to 12000, Cash to UPI with reference, reason &gt; Save</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
         <is>
-          <t>One row per student with pending fee: total, paid, pending, email goes to, last reminder; highest pending first</t>
+          <t>Same receipt number; amount and method corrected; pending reduced by 2000</t>
         </is>
       </c>
       <c r="F107" s="9" t="inlineStr">
@@ -4988,27 +4988,27 @@
       </c>
       <c r="B108" s="9" t="inlineStr">
         <is>
-          <t>Fee Reminders</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="C108" s="9" t="inlineStr">
         <is>
-          <t>Left student</t>
+          <t>Edit above the fee</t>
         </is>
       </c>
       <c r="D108" s="9" t="inlineStr">
         <is>
-          <t>Check out a student with pending fee</t>
+          <t>Edit a payment to more than the fee less the other payments</t>
         </is>
       </c>
       <c r="E108" s="9" t="inlineStr">
         <is>
-          <t>Still listed as '(left)'</t>
+          <t>Refused with the maximum allowed amount</t>
         </is>
       </c>
       <c r="F108" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G108" s="10" t="inlineStr">
@@ -5028,27 +5028,27 @@
       </c>
       <c r="B109" s="9" t="inlineStr">
         <is>
-          <t>Fee Reminders</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="C109" s="9" t="inlineStr">
         <is>
-          <t>Tick and send</t>
+          <t>Edit without changes</t>
         </is>
       </c>
       <c r="D109" s="9" t="inlineStr">
         <is>
-          <t>Tick 2 students &gt; Send Reminder (2) &gt; confirm</t>
+          <t>Edit &gt; Save without changing anything</t>
         </is>
       </c>
       <c r="E109" s="9" t="inlineStr">
         <is>
-          <t>2 emails with total, paid, pending and invoice PDF; copy to admin; Last reminder date shown</t>
+          <t>Message 'Nothing was changed'</t>
         </is>
       </c>
       <c r="F109" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G109" s="10" t="inlineStr">
@@ -5068,22 +5068,22 @@
       </c>
       <c r="B110" s="9" t="inlineStr">
         <is>
-          <t>Fee Reminders</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="C110" s="9" t="inlineStr">
         <is>
-          <t>Father, else mother</t>
+          <t>Delete with reason</t>
         </is>
       </c>
       <c r="D110" s="9" t="inlineStr">
         <is>
-          <t>Student without father email but with mother email</t>
+          <t>Payments &gt; Delete &gt; reason Entered twice &gt; Delete</t>
         </is>
       </c>
       <c r="E110" s="9" t="inlineStr">
         <is>
-          <t>Email to the mother; 'Mother: ...' shown</t>
+          <t>Payment removed; amount pending again</t>
         </is>
       </c>
       <c r="F110" s="9" t="inlineStr">
@@ -5108,27 +5108,27 @@
       </c>
       <c r="B111" s="9" t="inlineStr">
         <is>
-          <t>Fee Reminders</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="C111" s="9" t="inlineStr">
         <is>
-          <t>No parent email</t>
+          <t>Change history</t>
         </is>
       </c>
       <c r="D111" s="9" t="inlineStr">
         <is>
-          <t>Tick a student with no father or mother email &gt; Send</t>
+          <t>Payments &gt; Change History</t>
         </is>
       </c>
       <c r="E111" s="9" t="inlineStr">
         <is>
-          <t>Shown in red; listed as a problem; others sent</t>
+          <t>Every edit and delete with date, receipt, student, old and new values, reason; deletions in red</t>
         </is>
       </c>
       <c r="F111" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G111" s="10" t="inlineStr">
@@ -5153,22 +5153,22 @@
       </c>
       <c r="C112" s="9" t="inlineStr">
         <is>
-          <t>Select All / Clear</t>
+          <t>List</t>
         </is>
       </c>
       <c r="D112" s="9" t="inlineStr">
         <is>
-          <t>Select All, then Clear</t>
+          <t>Fee Reminders</t>
         </is>
       </c>
       <c r="E112" s="9" t="inlineStr">
         <is>
-          <t>All emailable students ticked, then none; button count updates</t>
+          <t>One row per student with pending fee: total, paid, pending, email goes to, last reminder; highest pending first</t>
         </is>
       </c>
       <c r="F112" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G112" s="10" t="inlineStr">
@@ -5193,22 +5193,22 @@
       </c>
       <c r="C113" s="9" t="inlineStr">
         <is>
-          <t>Preview</t>
+          <t>Left student</t>
         </is>
       </c>
       <c r="D113" s="9" t="inlineStr">
         <is>
-          <t>Select a student</t>
+          <t>Check out a student with pending fee</t>
         </is>
       </c>
       <c r="E113" s="9" t="inlineStr">
         <is>
-          <t>Preview shows To, subject and the text with that student's amounts</t>
+          <t>Still listed as '(left)'</t>
         </is>
       </c>
       <c r="F113" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G113" s="10" t="inlineStr">
@@ -5233,22 +5233,22 @@
       </c>
       <c r="C114" s="9" t="inlineStr">
         <is>
-          <t>Change text for this sending</t>
+          <t>Tick and send</t>
         </is>
       </c>
       <c r="D114" s="9" t="inlineStr">
         <is>
-          <t>Edit the message &gt; Send</t>
+          <t>Tick 2 students &gt; Send Reminder (2) &gt; confirm</t>
         </is>
       </c>
       <c r="E114" s="9" t="inlineStr">
         <is>
-          <t>Changed text sent; saved default unchanged</t>
+          <t>2 emails with total, paid, pending and invoice PDF; copy to admin; Last reminder date shown</t>
         </is>
       </c>
       <c r="F114" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G114" s="10" t="inlineStr">
@@ -5273,22 +5273,22 @@
       </c>
       <c r="C115" s="9" t="inlineStr">
         <is>
-          <t>Save as default</t>
+          <t>Father, else mother</t>
         </is>
       </c>
       <c r="D115" s="9" t="inlineStr">
         <is>
-          <t>Edit &gt; Save as Default; then Saved Text</t>
+          <t>Student without father email but with mother email</t>
         </is>
       </c>
       <c r="E115" s="9" t="inlineStr">
         <is>
-          <t>Text kept for next time; Saved Text reloads it</t>
+          <t>Email to the mother; 'Mother: ...' shown</t>
         </is>
       </c>
       <c r="F115" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G115" s="10" t="inlineStr">
@@ -5313,22 +5313,22 @@
       </c>
       <c r="C116" s="9" t="inlineStr">
         <is>
-          <t>Unknown field</t>
+          <t>No parent email</t>
         </is>
       </c>
       <c r="D116" s="9" t="inlineStr">
         <is>
-          <t>Type {Overdue} in the text &gt; Send or Save</t>
+          <t>Tick a student with no father or mother email &gt; Send</t>
         </is>
       </c>
       <c r="E116" s="9" t="inlineStr">
         <is>
-          <t>Error listing the available fields</t>
+          <t>Shown in red; listed as a problem; others sent</t>
         </is>
       </c>
       <c r="F116" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G116" s="10" t="inlineStr">
@@ -5353,22 +5353,22 @@
       </c>
       <c r="C117" s="9" t="inlineStr">
         <is>
-          <t>Never automatic</t>
+          <t>Select All / Clear</t>
         </is>
       </c>
       <c r="D117" s="9" t="inlineStr">
         <is>
-          <t>Leave the program open for a day</t>
+          <t>Select All, then Clear</t>
         </is>
       </c>
       <c r="E117" s="9" t="inlineStr">
         <is>
-          <t>No reminder is sent unless the admin clicks Send</t>
+          <t>All emailable students ticked, then none; button count updates</t>
         </is>
       </c>
       <c r="F117" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G117" s="10" t="inlineStr">
@@ -5393,22 +5393,22 @@
       </c>
       <c r="C118" s="9" t="inlineStr">
         <is>
-          <t>Record payment</t>
+          <t>Preview</t>
         </is>
       </c>
       <c r="D118" s="9" t="inlineStr">
         <is>
-          <t>Select a student &gt; Record Payment</t>
+          <t>Select a student</t>
         </is>
       </c>
       <c r="E118" s="9" t="inlineStr">
         <is>
-          <t>Payment recorded; amounts update</t>
+          <t>Preview shows To, subject and the text with that student's amounts</t>
         </is>
       </c>
       <c r="F118" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G118" s="10" t="inlineStr">
@@ -5433,17 +5433,17 @@
       </c>
       <c r="C119" s="9" t="inlineStr">
         <is>
-          <t>Export PDF</t>
+          <t>Change text for this sending</t>
         </is>
       </c>
       <c r="D119" s="9" t="inlineStr">
         <is>
-          <t>Export PDF</t>
+          <t>Edit the message &gt; Send</t>
         </is>
       </c>
       <c r="E119" s="9" t="inlineStr">
         <is>
-          <t>PDF of the list with totals and page numbers</t>
+          <t>Changed text sent; saved default unchanged</t>
         </is>
       </c>
       <c r="F119" s="9" t="inlineStr">
@@ -5468,27 +5468,27 @@
       </c>
       <c r="B120" s="9" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Fee Reminders</t>
         </is>
       </c>
       <c r="C120" s="9" t="inlineStr">
         <is>
-          <t>Test email</t>
+          <t>Save as default</t>
         </is>
       </c>
       <c r="D120" s="9" t="inlineStr">
         <is>
-          <t>Email Settings &gt; app password &gt; Send test to address &gt; Send Test Email</t>
+          <t>Edit &gt; Save as Default; then Saved Text</t>
         </is>
       </c>
       <c r="E120" s="9" t="inlineStr">
         <is>
-          <t>'Test email sent'; email arrives</t>
+          <t>Text kept for next time; Saved Text reloads it</t>
         </is>
       </c>
       <c r="F120" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G120" s="10" t="inlineStr">
@@ -5508,27 +5508,27 @@
       </c>
       <c r="B121" s="9" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Fee Reminders</t>
         </is>
       </c>
       <c r="C121" s="9" t="inlineStr">
         <is>
-          <t>Wrong app password</t>
+          <t>Unknown field</t>
         </is>
       </c>
       <c r="D121" s="9" t="inlineStr">
         <is>
-          <t>Enter a wrong app password &gt; Send Test Email</t>
+          <t>Type {Overdue} in the text &gt; Send or Save</t>
         </is>
       </c>
       <c r="E121" s="9" t="inlineStr">
         <is>
-          <t>Message 'Gmail did not accept the sender address and app password'</t>
+          <t>Error listing the available fields</t>
         </is>
       </c>
       <c r="F121" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G121" s="10" t="inlineStr">
@@ -5548,22 +5548,22 @@
       </c>
       <c r="B122" s="9" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Fee Reminders</t>
         </is>
       </c>
       <c r="C122" s="9" t="inlineStr">
         <is>
-          <t>No internet</t>
+          <t>Never automatic</t>
         </is>
       </c>
       <c r="D122" s="9" t="inlineStr">
         <is>
-          <t>Disconnect internet &gt; send</t>
+          <t>Leave the program open for a day</t>
         </is>
       </c>
       <c r="E122" s="9" t="inlineStr">
         <is>
-          <t>Message 'Could not connect to smtp.gmail.com'</t>
+          <t>No reminder is sent unless the admin clicks Send</t>
         </is>
       </c>
       <c r="F122" s="9" t="inlineStr">
@@ -5588,27 +5588,27 @@
       </c>
       <c r="B123" s="9" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Fee Reminders</t>
         </is>
       </c>
       <c r="C123" s="9" t="inlineStr">
         <is>
-          <t>Email invoice</t>
+          <t>Record payment</t>
         </is>
       </c>
       <c r="D123" s="9" t="inlineStr">
         <is>
-          <t>Invoices &gt; Email</t>
+          <t>Select a student &gt; Record Payment</t>
         </is>
       </c>
       <c r="E123" s="9" t="inlineStr">
         <is>
-          <t>Father (or mother) receives the invoice PDF with paid and pending; admin gets a copy</t>
+          <t>Payment recorded; amounts update</t>
         </is>
       </c>
       <c r="F123" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G123" s="10" t="inlineStr">
@@ -5628,27 +5628,27 @@
       </c>
       <c r="B124" s="9" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Fee Reminders</t>
         </is>
       </c>
       <c r="C124" s="9" t="inlineStr">
         <is>
-          <t>Email receipt</t>
+          <t>Export PDF</t>
         </is>
       </c>
       <c r="D124" s="9" t="inlineStr">
         <is>
-          <t>Payments &gt; Email Receipt</t>
+          <t>Export PDF</t>
         </is>
       </c>
       <c r="E124" s="9" t="inlineStr">
         <is>
-          <t>Father (or mother) receives the receipt PDF; admin copy</t>
+          <t>PDF of the list with totals and page numbers</t>
         </is>
       </c>
       <c r="F124" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G124" s="10" t="inlineStr">
@@ -5673,22 +5673,22 @@
       </c>
       <c r="C125" s="9" t="inlineStr">
         <is>
-          <t>Edit email text</t>
+          <t>Test email</t>
         </is>
       </c>
       <c r="D125" s="9" t="inlineStr">
         <is>
-          <t>Edit Invoice email subject &gt; Save &gt; send</t>
+          <t>Email Settings &gt; app password &gt; Send test to address &gt; Send Test Email</t>
         </is>
       </c>
       <c r="E125" s="9" t="inlineStr">
         <is>
-          <t>New subject used; Restore Default works</t>
+          <t>'Test email sent'; email arrives</t>
         </is>
       </c>
       <c r="F125" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G125" s="10" t="inlineStr">
@@ -5713,22 +5713,22 @@
       </c>
       <c r="C126" s="9" t="inlineStr">
         <is>
-          <t>Unknown field</t>
+          <t>Wrong app password</t>
         </is>
       </c>
       <c r="D126" s="9" t="inlineStr">
         <is>
-          <t>Type {ReceiptNo} in Receipt email &gt; Save</t>
+          <t>Enter a wrong app password &gt; Send Test Email</t>
         </is>
       </c>
       <c r="E126" s="9" t="inlineStr">
         <is>
-          <t>Error listing the available fields</t>
+          <t>Message 'Gmail did not accept the sender address and app password'</t>
         </is>
       </c>
       <c r="F126" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G126" s="10" t="inlineStr">
@@ -5753,17 +5753,17 @@
       </c>
       <c r="C127" s="9" t="inlineStr">
         <is>
-          <t>Email history</t>
+          <t>No internet</t>
         </is>
       </c>
       <c r="D127" s="9" t="inlineStr">
         <is>
-          <t>Email Settings &gt; Email history</t>
+          <t>Disconnect internet &gt; send</t>
         </is>
       </c>
       <c r="E127" s="9" t="inlineStr">
         <is>
-          <t>All sent and failed emails; failed in red with reason</t>
+          <t>Message 'Could not connect to smtp.gmail.com'</t>
         </is>
       </c>
       <c r="F127" s="9" t="inlineStr">
@@ -5793,22 +5793,22 @@
       </c>
       <c r="C128" s="9" t="inlineStr">
         <is>
-          <t>Not set up</t>
+          <t>Email invoice</t>
         </is>
       </c>
       <c r="D128" s="9" t="inlineStr">
         <is>
-          <t>Send an email before entering the app password</t>
+          <t>Invoices &gt; Email</t>
         </is>
       </c>
       <c r="E128" s="9" t="inlineStr">
         <is>
-          <t>Message to set up Email Settings first</t>
+          <t>Father (or mother) receives the invoice PDF with paid and pending; admin gets a copy</t>
         </is>
       </c>
       <c r="F128" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G128" s="10" t="inlineStr">
@@ -5828,22 +5828,22 @@
       </c>
       <c r="B129" s="9" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C129" s="9" t="inlineStr">
         <is>
-          <t>Figures</t>
+          <t>Email receipt</t>
         </is>
       </c>
       <c r="D129" s="9" t="inlineStr">
         <is>
-          <t>Compare with Students, Rooms, Invoices, Payments, Fee Reminders</t>
+          <t>Payments &gt; Email Receipt</t>
         </is>
       </c>
       <c r="E129" s="9" t="inlineStr">
         <is>
-          <t>Students, beds, fees this year, received this month and year, pending match</t>
+          <t>Father (or mother) receives the receipt PDF; admin copy</t>
         </is>
       </c>
       <c r="F129" s="9" t="inlineStr">
@@ -5868,22 +5868,22 @@
       </c>
       <c r="B130" s="9" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C130" s="9" t="inlineStr">
         <is>
-          <t>Chart</t>
+          <t>Edit email text</t>
         </is>
       </c>
       <c r="D130" s="9" t="inlineStr">
         <is>
-          <t>Record a payment today &gt; reopen Dashboard</t>
+          <t>Edit Invoice email subject &gt; Save &gt; send</t>
         </is>
       </c>
       <c r="E130" s="9" t="inlineStr">
         <is>
-          <t>Current month bar and Received increase; hover shows exact amount</t>
+          <t>New subject used; Restore Default works</t>
         </is>
       </c>
       <c r="F130" s="9" t="inlineStr">
@@ -5908,22 +5908,22 @@
       </c>
       <c r="B131" s="9" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C131" s="9" t="inlineStr">
         <is>
-          <t>Lists</t>
+          <t>Unknown field</t>
         </is>
       </c>
       <c r="D131" s="9" t="inlineStr">
         <is>
-          <t>Check the three lists</t>
+          <t>Type {ReceiptNo} in Receipt email &gt; Save</t>
         </is>
       </c>
       <c r="E131" s="9" t="inlineStr">
         <is>
-          <t>5 highest pending fees, latest payments, latest check-ins</t>
+          <t>Error listing the available fields</t>
         </is>
       </c>
       <c r="F131" s="9" t="inlineStr">
@@ -5948,22 +5948,22 @@
       </c>
       <c r="B132" s="9" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C132" s="9" t="inlineStr">
         <is>
-          <t>Other hostel</t>
+          <t>Email history</t>
         </is>
       </c>
       <c r="D132" s="9" t="inlineStr">
         <is>
-          <t>Switch hostel</t>
+          <t>Email Settings &gt; Email history</t>
         </is>
       </c>
       <c r="E132" s="9" t="inlineStr">
         <is>
-          <t>All figures change to that hostel</t>
+          <t>All sent and failed emails; failed in red with reason</t>
         </is>
       </c>
       <c r="F132" s="9" t="inlineStr">
@@ -5988,27 +5988,27 @@
       </c>
       <c r="B133" s="9" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C133" s="9" t="inlineStr">
         <is>
-          <t>Student list</t>
+          <t>Not set up</t>
         </is>
       </c>
       <c r="D133" s="9" t="inlineStr">
         <is>
-          <t>Reports &gt; Student list &gt; Active &gt; Show</t>
+          <t>Send an email before entering the app password</t>
         </is>
       </c>
       <c r="E133" s="9" t="inlineStr">
         <is>
-          <t>Active students with masked Aadhaar; total count</t>
+          <t>Message to set up Email Settings first</t>
         </is>
       </c>
       <c r="F133" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G133" s="10" t="inlineStr">
@@ -6028,22 +6028,22 @@
       </c>
       <c r="B134" s="9" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C134" s="9" t="inlineStr">
         <is>
-          <t>Room occupancy</t>
+          <t>Figures</t>
         </is>
       </c>
       <c r="D134" s="9" t="inlineStr">
         <is>
-          <t>Room occupancy &gt; Show</t>
+          <t>Compare with Students, Rooms, Invoices, Payments, Fee Reminders</t>
         </is>
       </c>
       <c r="E134" s="9" t="inlineStr">
         <is>
-          <t>Each room, beds, occupied, free, students (no rent); totals match Rooms screen</t>
+          <t>Students, beds, fees this year, received this month and year, pending match</t>
         </is>
       </c>
       <c r="F134" s="9" t="inlineStr">
@@ -6068,27 +6068,27 @@
       </c>
       <c r="B135" s="9" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C135" s="9" t="inlineStr">
         <is>
-          <t>Payments received</t>
+          <t>Chart</t>
         </is>
       </c>
       <c r="D135" s="9" t="inlineStr">
         <is>
-          <t>Dates of the month &gt; Show</t>
+          <t>Record a payment today &gt; reopen Dashboard</t>
         </is>
       </c>
       <c r="E135" s="9" t="inlineStr">
         <is>
-          <t>Payments with a total per day, per method and grand total</t>
+          <t>Current month bar and Received increase; hover shows exact amount</t>
         </is>
       </c>
       <c r="F135" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G135" s="10" t="inlineStr">
@@ -6108,27 +6108,27 @@
       </c>
       <c r="B136" s="9" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C136" s="9" t="inlineStr">
         <is>
-          <t>Fees report</t>
+          <t>Lists</t>
         </is>
       </c>
       <c r="D136" s="9" t="inlineStr">
         <is>
-          <t>Fees (invoices) &gt; Year 2026-27, status Unpaid</t>
+          <t>Check the three lists</t>
         </is>
       </c>
       <c r="E136" s="9" t="inlineStr">
         <is>
-          <t>Only unpaid fees of that year with rent, transport, total, paid, pending; totals</t>
+          <t>5 highest pending fees, latest payments, latest check-ins</t>
         </is>
       </c>
       <c r="F136" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G136" s="10" t="inlineStr">
@@ -6148,22 +6148,22 @@
       </c>
       <c r="B137" s="9" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C137" s="9" t="inlineStr">
         <is>
-          <t>Export PDF</t>
+          <t>Other hostel</t>
         </is>
       </c>
       <c r="D137" s="9" t="inlineStr">
         <is>
-          <t>Any report &gt; Export PDF</t>
+          <t>Switch hostel</t>
         </is>
       </c>
       <c r="E137" s="9" t="inlineStr">
         <is>
-          <t>PDF opens, headings on every page, page numbers</t>
+          <t>All figures change to that hostel</t>
         </is>
       </c>
       <c r="F137" s="9" t="inlineStr">
@@ -6193,22 +6193,22 @@
       </c>
       <c r="C138" s="9" t="inlineStr">
         <is>
-          <t>Export Excel</t>
+          <t>Student list</t>
         </is>
       </c>
       <c r="D138" s="9" t="inlineStr">
         <is>
-          <t>Any report &gt; Export Excel</t>
+          <t>Reports &gt; Student list &gt; Active &gt; Show</t>
         </is>
       </c>
       <c r="E138" s="9" t="inlineStr">
         <is>
-          <t>Excel opens; amounts are numbers in rupees, dates are dates, filters work</t>
+          <t>Active students with masked Aadhaar; total count</t>
         </is>
       </c>
       <c r="F138" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G138" s="10" t="inlineStr">
@@ -6233,22 +6233,22 @@
       </c>
       <c r="C139" s="9" t="inlineStr">
         <is>
-          <t>Wrong dates</t>
+          <t>Room occupancy</t>
         </is>
       </c>
       <c r="D139" s="9" t="inlineStr">
         <is>
-          <t>From after To</t>
+          <t>Room occupancy &gt; Show</t>
         </is>
       </c>
       <c r="E139" s="9" t="inlineStr">
         <is>
-          <t>Error message</t>
+          <t>Each room, beds, occupied, free, students (no rent); totals match Rooms screen</t>
         </is>
       </c>
       <c r="F139" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G139" s="10" t="inlineStr">
@@ -6273,22 +6273,22 @@
       </c>
       <c r="C140" s="9" t="inlineStr">
         <is>
-          <t>Pending fees report</t>
+          <t>Payments received</t>
         </is>
       </c>
       <c r="D140" s="9" t="inlineStr">
         <is>
-          <t>Pending fees &gt; Show</t>
+          <t>Dates of the month &gt; Show</t>
         </is>
       </c>
       <c r="E140" s="9" t="inlineStr">
         <is>
-          <t>Student lines with total, paid, pending, then their invoices</t>
+          <t>Payments with a total per day, per method and grand total</t>
         </is>
       </c>
       <c r="F140" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G140" s="10" t="inlineStr">
@@ -6308,27 +6308,27 @@
       </c>
       <c r="B141" s="9" t="inlineStr">
         <is>
-          <t>Backup / Restore</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C141" s="9" t="inlineStr">
         <is>
-          <t>Backup now</t>
+          <t>Fees report</t>
         </is>
       </c>
       <c r="D141" s="9" t="inlineStr">
         <is>
-          <t>Backup / Restore &gt; Backup Now</t>
+          <t>Fees (invoices) &gt; Year 2026-27, status Unpaid</t>
         </is>
       </c>
       <c r="E141" s="9" t="inlineStr">
         <is>
-          <t>Zip in Backups listed as 'Backup Now'; contains database, photos, documents</t>
+          <t>Only unpaid fees of that year with rent, transport, total, paid, pending; totals</t>
         </is>
       </c>
       <c r="F141" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G141" s="10" t="inlineStr">
@@ -6348,27 +6348,27 @@
       </c>
       <c r="B142" s="9" t="inlineStr">
         <is>
-          <t>Backup / Restore</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C142" s="9" t="inlineStr">
         <is>
-          <t>Daily automatic backup</t>
+          <t>Export PDF</t>
         </is>
       </c>
       <c r="D142" s="9" t="inlineStr">
         <is>
-          <t>Close the program (first time today)</t>
+          <t>Any report &gt; Export PDF</t>
         </is>
       </c>
       <c r="E142" s="9" t="inlineStr">
         <is>
-          <t>Automatic backup made; only one per day</t>
+          <t>PDF opens, headings on every page, page numbers</t>
         </is>
       </c>
       <c r="F142" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G142" s="10" t="inlineStr">
@@ -6388,22 +6388,22 @@
       </c>
       <c r="B143" s="9" t="inlineStr">
         <is>
-          <t>Backup / Restore</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C143" s="9" t="inlineStr">
         <is>
-          <t>Second copy folder</t>
+          <t>Export Excel</t>
         </is>
       </c>
       <c r="D143" s="9" t="inlineStr">
         <is>
-          <t>Choose a USB / Google Drive folder &gt; Backup Now</t>
+          <t>Any report &gt; Export Excel</t>
         </is>
       </c>
       <c r="E143" s="9" t="inlineStr">
         <is>
-          <t>Zip also in that folder</t>
+          <t>Excel opens; amounts are numbers in rupees, dates are dates, filters work</t>
         </is>
       </c>
       <c r="F143" s="9" t="inlineStr">
@@ -6428,22 +6428,22 @@
       </c>
       <c r="B144" s="9" t="inlineStr">
         <is>
-          <t>Backup / Restore</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C144" s="9" t="inlineStr">
         <is>
-          <t>Second folder missing</t>
+          <t>Wrong dates</t>
         </is>
       </c>
       <c r="D144" s="9" t="inlineStr">
         <is>
-          <t>Remove the USB &gt; Backup Now</t>
+          <t>From after To</t>
         </is>
       </c>
       <c r="E144" s="9" t="inlineStr">
         <is>
-          <t>Backup made; message that the second copy failed</t>
+          <t>Error message</t>
         </is>
       </c>
       <c r="F144" s="9" t="inlineStr">
@@ -6468,27 +6468,27 @@
       </c>
       <c r="B145" s="9" t="inlineStr">
         <is>
-          <t>Backup / Restore</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="C145" s="9" t="inlineStr">
         <is>
-          <t>Restore</t>
+          <t>Pending fees report</t>
         </is>
       </c>
       <c r="D145" s="9" t="inlineStr">
         <is>
-          <t>Add a test hostel &gt; Restore an older backup &gt; confirm</t>
+          <t>Pending fees &gt; Show</t>
         </is>
       </c>
       <c r="E145" s="9" t="inlineStr">
         <is>
-          <t>Program restarts; test hostel gone; 'Before a restore' backup created</t>
+          <t>Student lines with total, paid, pending, then their invoices</t>
         </is>
       </c>
       <c r="F145" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G145" s="10" t="inlineStr">
@@ -6513,22 +6513,22 @@
       </c>
       <c r="C146" s="9" t="inlineStr">
         <is>
-          <t>Undo restore</t>
+          <t>Backup now</t>
         </is>
       </c>
       <c r="D146" s="9" t="inlineStr">
         <is>
-          <t>Restore the 'Before a restore' backup</t>
+          <t>Backup / Restore &gt; Backup Now</t>
         </is>
       </c>
       <c r="E146" s="9" t="inlineStr">
         <is>
-          <t>Data from before the restore is back</t>
+          <t>Zip in Backups listed as 'Backup Now'; contains database, photos, documents</t>
         </is>
       </c>
       <c r="F146" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G146" s="10" t="inlineStr">
@@ -6553,22 +6553,22 @@
       </c>
       <c r="C147" s="9" t="inlineStr">
         <is>
-          <t>Wrong file</t>
+          <t>Daily automatic backup</t>
         </is>
       </c>
       <c r="D147" s="9" t="inlineStr">
         <is>
-          <t>Restore From File &gt; choose a non-backup zip</t>
+          <t>Close the program (first time today)</t>
         </is>
       </c>
       <c r="E147" s="9" t="inlineStr">
         <is>
-          <t>Clear error; nothing changed</t>
+          <t>Automatic backup made; only one per day</t>
         </is>
       </c>
       <c r="F147" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G147" s="10" t="inlineStr">
@@ -6588,22 +6588,22 @@
       </c>
       <c r="B148" s="9" t="inlineStr">
         <is>
-          <t>Application Settings</t>
+          <t>Backup / Restore</t>
         </is>
       </c>
       <c r="C148" s="9" t="inlineStr">
         <is>
-          <t>Database check</t>
+          <t>Second copy folder</t>
         </is>
       </c>
       <c r="D148" s="9" t="inlineStr">
         <is>
-          <t>Application Settings &gt; Test Database</t>
+          <t>Choose a USB / Google Drive folder &gt; Backup Now</t>
         </is>
       </c>
       <c r="E148" s="9" t="inlineStr">
         <is>
-          <t>All steps pass</t>
+          <t>Zip also in that folder</t>
         </is>
       </c>
       <c r="F148" s="9" t="inlineStr">
@@ -6628,22 +6628,22 @@
       </c>
       <c r="B149" s="9" t="inlineStr">
         <is>
-          <t>Application Settings</t>
+          <t>Backup / Restore</t>
         </is>
       </c>
       <c r="C149" s="9" t="inlineStr">
         <is>
-          <t>User guide</t>
+          <t>Second folder missing</t>
         </is>
       </c>
       <c r="D149" s="9" t="inlineStr">
         <is>
-          <t>Application Settings &gt; User Guide</t>
+          <t>Remove the USB &gt; Backup Now</t>
         </is>
       </c>
       <c r="E149" s="9" t="inlineStr">
         <is>
-          <t>User guide opens</t>
+          <t>Backup made; message that the second copy failed</t>
         </is>
       </c>
       <c r="F149" s="9" t="inlineStr">
@@ -6668,27 +6668,27 @@
       </c>
       <c r="B150" s="9" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Backup / Restore</t>
         </is>
       </c>
       <c r="C150" s="9" t="inlineStr">
         <is>
-          <t>Menu fits screen</t>
+          <t>Restore</t>
         </is>
       </c>
       <c r="D150" s="9" t="inlineStr">
         <is>
-          <t>Laptop 1366 x 768, maximised</t>
+          <t>Add a test hostel &gt; Restore an older backup &gt; confirm</t>
         </is>
       </c>
       <c r="E150" s="9" t="inlineStr">
         <is>
-          <t>No scroll bar in the left menu</t>
+          <t>Program restarts; test hostel gone; 'Before a restore' backup created</t>
         </is>
       </c>
       <c r="F150" s="9" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G150" s="10" t="inlineStr">
@@ -6708,22 +6708,22 @@
       </c>
       <c r="B151" s="9" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Backup / Restore</t>
         </is>
       </c>
       <c r="C151" s="9" t="inlineStr">
         <is>
-          <t>No technical errors shown</t>
+          <t>Undo restore</t>
         </is>
       </c>
       <c r="D151" s="9" t="inlineStr">
         <is>
-          <t>Cause errors (e.g. open the database in Access and save)</t>
+          <t>Restore the 'Before a restore' backup</t>
         </is>
       </c>
       <c r="E151" s="9" t="inlineStr">
         <is>
-          <t>Friendly message; details in Logs</t>
+          <t>Data from before the restore is back</t>
         </is>
       </c>
       <c r="F151" s="9" t="inlineStr">
@@ -6748,27 +6748,27 @@
       </c>
       <c r="B152" s="9" t="inlineStr">
         <is>
-          <t>Uninstall</t>
+          <t>Backup / Restore</t>
         </is>
       </c>
       <c r="C152" s="9" t="inlineStr">
         <is>
-          <t>Uninstall keeps data</t>
+          <t>Wrong file</t>
         </is>
       </c>
       <c r="D152" s="9" t="inlineStr">
         <is>
-          <t>Settings &gt; Apps &gt; Uninstall</t>
+          <t>Restore From File &gt; choose a non-backup zip</t>
         </is>
       </c>
       <c r="E152" s="9" t="inlineStr">
         <is>
-          <t>Program removed; Database, Photos, Documents, Invoices, Receipts, Reports, Agreements, Backups kept</t>
+          <t>Clear error; nothing changed</t>
         </is>
       </c>
       <c r="F152" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G152" s="10" t="inlineStr">
@@ -6788,27 +6788,27 @@
       </c>
       <c r="B153" s="9" t="inlineStr">
         <is>
-          <t>Uninstall</t>
+          <t>Application Settings</t>
         </is>
       </c>
       <c r="C153" s="9" t="inlineStr">
         <is>
-          <t>Reinstall uses old data</t>
+          <t>Database check</t>
         </is>
       </c>
       <c r="D153" s="9" t="inlineStr">
         <is>
-          <t>Install again into C:\HostelManagement</t>
+          <t>Application Settings &gt; Test Database</t>
         </is>
       </c>
       <c r="E153" s="9" t="inlineStr">
         <is>
-          <t>All data is back</t>
+          <t>All steps pass</t>
         </is>
       </c>
       <c r="F153" s="9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G153" s="10" t="inlineStr">
@@ -6820,9 +6820,209 @@
       <c r="I153" s="11" t="inlineStr"/>
       <c r="J153" s="10" t="inlineStr"/>
     </row>
+    <row r="154">
+      <c r="A154" s="9" t="inlineStr">
+        <is>
+          <t>TC-153</t>
+        </is>
+      </c>
+      <c r="B154" s="9" t="inlineStr">
+        <is>
+          <t>Application Settings</t>
+        </is>
+      </c>
+      <c r="C154" s="9" t="inlineStr">
+        <is>
+          <t>User guide</t>
+        </is>
+      </c>
+      <c r="D154" s="9" t="inlineStr">
+        <is>
+          <t>Application Settings &gt; User Guide</t>
+        </is>
+      </c>
+      <c r="E154" s="9" t="inlineStr">
+        <is>
+          <t>User guide opens</t>
+        </is>
+      </c>
+      <c r="F154" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G154" s="10" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="H154" s="10" t="inlineStr"/>
+      <c r="I154" s="11" t="inlineStr"/>
+      <c r="J154" s="10" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="9" t="inlineStr">
+        <is>
+          <t>TC-154</t>
+        </is>
+      </c>
+      <c r="B155" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C155" s="9" t="inlineStr">
+        <is>
+          <t>Menu fits screen</t>
+        </is>
+      </c>
+      <c r="D155" s="9" t="inlineStr">
+        <is>
+          <t>Laptop 1366 x 768, maximised</t>
+        </is>
+      </c>
+      <c r="E155" s="9" t="inlineStr">
+        <is>
+          <t>No scroll bar in the left menu</t>
+        </is>
+      </c>
+      <c r="F155" s="9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G155" s="10" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="H155" s="10" t="inlineStr"/>
+      <c r="I155" s="11" t="inlineStr"/>
+      <c r="J155" s="10" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="9" t="inlineStr">
+        <is>
+          <t>TC-155</t>
+        </is>
+      </c>
+      <c r="B156" s="9" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C156" s="9" t="inlineStr">
+        <is>
+          <t>No technical errors shown</t>
+        </is>
+      </c>
+      <c r="D156" s="9" t="inlineStr">
+        <is>
+          <t>Cause errors (e.g. open the database in Access and save)</t>
+        </is>
+      </c>
+      <c r="E156" s="9" t="inlineStr">
+        <is>
+          <t>Friendly message; details in Logs</t>
+        </is>
+      </c>
+      <c r="F156" s="9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G156" s="10" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="H156" s="10" t="inlineStr"/>
+      <c r="I156" s="11" t="inlineStr"/>
+      <c r="J156" s="10" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="9" t="inlineStr">
+        <is>
+          <t>TC-156</t>
+        </is>
+      </c>
+      <c r="B157" s="9" t="inlineStr">
+        <is>
+          <t>Uninstall</t>
+        </is>
+      </c>
+      <c r="C157" s="9" t="inlineStr">
+        <is>
+          <t>Uninstall keeps data</t>
+        </is>
+      </c>
+      <c r="D157" s="9" t="inlineStr">
+        <is>
+          <t>Settings &gt; Apps &gt; Uninstall</t>
+        </is>
+      </c>
+      <c r="E157" s="9" t="inlineStr">
+        <is>
+          <t>Program removed; Database, Photos, Documents, Invoices, Receipts, Reports, Agreements, Backups kept</t>
+        </is>
+      </c>
+      <c r="F157" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G157" s="10" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="H157" s="10" t="inlineStr"/>
+      <c r="I157" s="11" t="inlineStr"/>
+      <c r="J157" s="10" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="9" t="inlineStr">
+        <is>
+          <t>TC-157</t>
+        </is>
+      </c>
+      <c r="B158" s="9" t="inlineStr">
+        <is>
+          <t>Uninstall</t>
+        </is>
+      </c>
+      <c r="C158" s="9" t="inlineStr">
+        <is>
+          <t>Reinstall uses old data</t>
+        </is>
+      </c>
+      <c r="D158" s="9" t="inlineStr">
+        <is>
+          <t>Install again into C:\HostelManagement</t>
+        </is>
+      </c>
+      <c r="E158" s="9" t="inlineStr">
+        <is>
+          <t>All data is back</t>
+        </is>
+      </c>
+      <c r="F158" s="9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G158" s="10" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="H158" s="10" t="inlineStr"/>
+      <c r="I158" s="11" t="inlineStr"/>
+      <c r="J158" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J153"/>
-  <conditionalFormatting sqref="G2:G153">
+  <autoFilter ref="A1:J158"/>
+  <conditionalFormatting sqref="G2:G158">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -6834,7 +7034,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G153" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not run,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7699,23 +7899,23 @@
         </is>
       </c>
       <c r="B2" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A2)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A2)</f>
         <v/>
       </c>
       <c r="C2" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A2,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A2,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D2" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A2,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A2,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E2" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A2,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A2,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F2" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A2,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A2,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G2" s="14">
@@ -7730,23 +7930,23 @@
         </is>
       </c>
       <c r="B3" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A3)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A3)</f>
         <v/>
       </c>
       <c r="C3" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A3,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A3,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A3,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A3,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E3" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A3,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A3,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F3" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A3,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A3,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G3" s="14">
@@ -7761,23 +7961,23 @@
         </is>
       </c>
       <c r="B4" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A4)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A4)</f>
         <v/>
       </c>
       <c r="C4" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A4,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A4,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A4,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A4,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E4" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A4,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A4,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F4" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A4,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A4,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G4" s="14">
@@ -7792,23 +7992,23 @@
         </is>
       </c>
       <c r="B5" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A5)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A5)</f>
         <v/>
       </c>
       <c r="C5" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A5,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A5,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A5,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A5,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E5" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A5,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A5,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F5" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A5,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A5,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G5" s="14">
@@ -7823,23 +8023,23 @@
         </is>
       </c>
       <c r="B6" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A6)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A6)</f>
         <v/>
       </c>
       <c r="C6" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A6,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A6,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D6" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A6,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A6,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E6" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A6,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A6,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F6" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A6,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A6,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G6" s="14">
@@ -7854,23 +8054,23 @@
         </is>
       </c>
       <c r="B7" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A7)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A7)</f>
         <v/>
       </c>
       <c r="C7" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A7,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A7,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D7" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A7,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A7,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E7" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A7,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A7,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F7" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A7,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A7,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G7" s="14">
@@ -7885,23 +8085,23 @@
         </is>
       </c>
       <c r="B8" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A8)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A8)</f>
         <v/>
       </c>
       <c r="C8" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A8,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A8,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D8" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A8,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A8,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E8" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A8,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A8,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F8" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A8,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A8,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G8" s="14">
@@ -7916,23 +8116,23 @@
         </is>
       </c>
       <c r="B9" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A9)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A9)</f>
         <v/>
       </c>
       <c r="C9" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A9,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A9,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D9" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A9,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A9,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E9" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A9,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A9,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F9" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A9,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A9,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G9" s="14">
@@ -7947,23 +8147,23 @@
         </is>
       </c>
       <c r="B10" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A10)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A10)</f>
         <v/>
       </c>
       <c r="C10" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A10,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A10,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D10" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A10,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A10,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E10" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A10,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A10,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F10" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A10,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A10,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G10" s="14">
@@ -7978,23 +8178,23 @@
         </is>
       </c>
       <c r="B11" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A11)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A11)</f>
         <v/>
       </c>
       <c r="C11" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A11,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A11,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D11" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A11,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A11,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E11" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A11,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A11,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F11" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A11,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A11,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G11" s="14">
@@ -8009,23 +8209,23 @@
         </is>
       </c>
       <c r="B12" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A12)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A12)</f>
         <v/>
       </c>
       <c r="C12" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A12,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A12,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D12" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A12,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A12,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E12" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A12,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A12,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F12" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A12,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A12,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G12" s="14">
@@ -8040,23 +8240,23 @@
         </is>
       </c>
       <c r="B13" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A13)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A13)</f>
         <v/>
       </c>
       <c r="C13" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A13,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A13,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A13,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A13,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A13,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A13,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F13" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A13,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A13,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G13" s="14">
@@ -8071,23 +8271,23 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A14)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A14)</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A14,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A14,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A14,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A14,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A14,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A14,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F14" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A14,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A14,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G14" s="14">
@@ -8102,23 +8302,23 @@
         </is>
       </c>
       <c r="B15" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A15)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A15)</f>
         <v/>
       </c>
       <c r="C15" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A15,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A15,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A15,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A15,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A15,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A15,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F15" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A15,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A15,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G15" s="14">
@@ -8133,23 +8333,23 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A16)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A16)</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A16,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A16,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A16,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A16,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A16,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A16,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F16" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A16,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A16,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G16" s="14">
@@ -8164,23 +8364,23 @@
         </is>
       </c>
       <c r="B17" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A17)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A17)</f>
         <v/>
       </c>
       <c r="C17" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A17,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A17,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A17,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A17,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A17,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A17,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F17" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A17,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A17,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G17" s="14">
@@ -8195,23 +8395,23 @@
         </is>
       </c>
       <c r="B18" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A18)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A18)</f>
         <v/>
       </c>
       <c r="C18" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A18,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A18,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A18,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A18,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A18,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A18,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F18" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A18,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A18,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G18" s="14">
@@ -8226,23 +8426,23 @@
         </is>
       </c>
       <c r="B19" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A19)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A19)</f>
         <v/>
       </c>
       <c r="C19" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A19,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A19,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A19,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A19,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A19,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A19,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F19" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A19,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A19,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G19" s="14">
@@ -8257,23 +8457,23 @@
         </is>
       </c>
       <c r="B20" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A20)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A20)</f>
         <v/>
       </c>
       <c r="C20" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A20,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A20,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A20,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A20,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A20,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A20,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F20" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A20,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A20,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G20" s="14">
@@ -8288,23 +8488,23 @@
         </is>
       </c>
       <c r="B21" s="13">
-        <f>COUNTIF('Test Cases'!$B$2:$B$153,A21)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$158,A21)</f>
         <v/>
       </c>
       <c r="C21" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A21,'Test Cases'!$G$2:$G$153,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A21,'Test Cases'!$G$2:$G$158,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A21,'Test Cases'!$G$2:$G$153,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A21,'Test Cases'!$G$2:$G$158,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A21,'Test Cases'!$G$2:$G$153,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A21,'Test Cases'!$G$2:$G$158,"Blocked")</f>
         <v/>
       </c>
       <c r="F21" s="13">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$153,$A21,'Test Cases'!$G$2:$G$153,"Not run")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$158,$A21,'Test Cases'!$G$2:$G$158,"Not run")</f>
         <v/>
       </c>
       <c r="G21" s="14">

</xml_diff>